<commit_message>
Update anatomy source data and references
</commit_message>
<xml_diff>
--- a/data/untere-extremitaet -+ fuß komplett umgewandelt .xlsx
+++ b/data/untere-extremitaet -+ fuß komplett umgewandelt .xlsx
@@ -717,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA59"/>
+  <dimension ref="A1:AA58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col width="28" customWidth="1" style="30" min="1" max="1"/>
@@ -3794,7 +3794,7 @@
       <c r="V34" s="5" t="n"/>
       <c r="W34" s="5" t="inlineStr">
         <is>
-          <t>Beugt das Knie (Flexion in der Art. genus) und entriegelt die Vollextension durch Innenrotation des Unterschenkels; zieht den lateralen Meniskus nach dorsal</t>
+          <t>Leitet die Kniebeugung ein, rotiert den Unterschenkel nach innen und entlastet den Außenmeniskus</t>
         </is>
       </c>
       <c r="X34" s="5" t="inlineStr">
@@ -4066,7 +4066,7 @@
       </c>
       <c r="F38" s="14" t="inlineStr">
         <is>
-          <t>Fehlt bei etwa 15 % der Bevölkerung; seine dünne Sehne ist als Transplantatmaterial beliebt (z.B. für Bandrekonstruktionen); klinisch selten symptomatisch</t>
+          <t>Der Muskel fehlt bei vielen Menschen ganz; meist bleibt das ohne Beschwerden, die Sehne wird aber teils als Transplantat genutzt</t>
         </is>
       </c>
       <c r="G38" s="14" t="inlineStr">
@@ -5075,7 +5075,7 @@
       </c>
       <c r="F49" s="14" t="inlineStr">
         <is>
-          <t>Korrigiert den durch den Zug des M. flexor digitorum longus entstehenden schrägen Zugvektor; erst durch ihn erfolgt eine achsengerechte Zehenflexion</t>
+          <t>Verbessert die Kraftübertragung auf die Kleinzehen; Schwäche macht die plantare Zehenbeugung weniger sauber</t>
         </is>
       </c>
       <c r="G49" s="14" t="inlineStr">
@@ -5120,7 +5120,7 @@
       <c r="V49" s="14" t="n"/>
       <c r="W49" s="14" t="inlineStr">
         <is>
-          <t>Richtet den Zugvektor des M. flexor digitorum longus auf die Zehenlängsachse aus; unterstützt die Beugung der Zehen II–V</t>
+          <t>Richtet die Zugrichtung des langen Zehenbeugers aus und unterstützt das Beugen der Kleinzehen</t>
         </is>
       </c>
       <c r="X49" s="14" t="inlineStr">
@@ -5484,7 +5484,7 @@
       <c r="V53" s="14" t="n"/>
       <c r="W53" s="14" t="inlineStr">
         <is>
-          <t>Streckt die Großzehe im MTP-Gelenk; unterstützt den M. extensor hallucis longus bei der Großzehenstreckung</t>
+          <t>Streckt die Großzehe im Grundgelenk und unterstützt die lange Strecksehne</t>
         </is>
       </c>
       <c r="X53" s="14" t="inlineStr">
@@ -5885,186 +5885,95 @@
       <c r="AA57" s="14" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>M. opponens digiti minimi</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>M. abductor digiti minimi</t>
+        </is>
+      </c>
+      <c r="B58" s="13" t="inlineStr">
         <is>
           <t>untere-extremitaet</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="13" t="inlineStr">
         <is>
           <t>fuss</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>fuss,kleinzehenabduktion,kleinzehenflexion,kurze-fussmuskulatur,fusssohle</t>
-        </is>
-      </c>
-      <c r="E58" t="n">
-        <v>3</v>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Wird oft nur als tiefer Anteil des M. flexor digiti minimi brevis beschrieben und daher in Lehrwerken nicht immer separat aufgeführt; funktionell trägt er zur Stabilisierung des lateralen Fußrandes bei</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
+      <c r="D58" s="13" t="inlineStr">
+        <is>
+          <t>fuss,kleinzehenabduktion,kurze-fussmuskulatur,fusssohle</t>
+        </is>
+      </c>
+      <c r="E58" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="13" t="inlineStr">
+        <is>
+          <t>Bursitis am Tuber calcanei lateral und der sog. Tailor's bunion (Prominenz des fünften Mittelfußköpfchens) gehen häufig mit Reizung des Abductor digiti minimi einher</t>
+        </is>
+      </c>
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>Am lateralen Fußrand deutlich tastbar; der Muskelbauch ist von Ferse bis Kleinzehenbasis als prominenter Wulst zu verfolgen</t>
+        </is>
+      </c>
+      <c r="H58" s="13" t="inlineStr">
         <is>
           <t>MTP Zeh V</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="I58" s="13" t="inlineStr">
         <is>
           <t>Zeh V: Flexion und Abduktion des MTP-Gelenks</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>N. tibialis (N. plantaris lateralis), S2, S3</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>muscle_opponens_digiti_minimi_caudal_1.jpg</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>Lig. plantare longum</t>
-        </is>
-      </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>Basis des Os metatarsale V</t>
-        </is>
-      </c>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t>Sehnenscheide des M. fibularis longus</t>
-        </is>
-      </c>
-      <c r="T58" t="inlineStr">
-        <is>
-          <t>Lateraler Rand des Os metatarsale V</t>
-        </is>
-      </c>
-      <c r="W58" t="inlineStr">
-        <is>
-          <t>Unterstützt Flexion und Abduktion der Kleinzehe und stabilisiert das laterale Längsgewölbe des Fußes</t>
-        </is>
-      </c>
-      <c r="X58" t="inlineStr">
+      <c r="J58" s="13" t="inlineStr">
+        <is>
+          <t>N. tibialis (N. plantaris lateralis)</t>
+        </is>
+      </c>
+      <c r="K58" s="13" t="n"/>
+      <c r="L58" s="13" t="n"/>
+      <c r="M58" s="13" t="inlineStr">
+        <is>
+          <t>Tuber calcanei (Proc. lateralis) und Lig. plantare longum</t>
+        </is>
+      </c>
+      <c r="N58" s="13" t="n"/>
+      <c r="O58" s="13" t="n"/>
+      <c r="P58" s="13" t="n"/>
+      <c r="Q58" s="13" t="n"/>
+      <c r="R58" s="13" t="n"/>
+      <c r="S58" s="13" t="n"/>
+      <c r="T58" s="13" t="inlineStr">
+        <is>
+          <t>Zeh V, Tuberositas ossis metatarsalis V und proximale Phalanx (laterale Seite)</t>
+        </is>
+      </c>
+      <c r="U58" s="13" t="n"/>
+      <c r="V58" s="13" t="n"/>
+      <c r="W58" s="13" t="inlineStr">
+        <is>
+          <t>Abduziert und beugt die Kleinzehe im MTP-Gelenk; stabilisiert den lateralen Fußrand</t>
+        </is>
+      </c>
+      <c r="X58" s="13" t="inlineStr">
         <is>
           <t>BodyParts3D, © DBCLS</t>
         </is>
       </c>
-      <c r="Y58" t="inlineStr">
+      <c r="Y58" s="13" t="inlineStr">
         <is>
           <t>CC BY 4.0</t>
         </is>
       </c>
-      <c r="Z58" t="inlineStr">
+      <c r="Z58" s="13" t="inlineStr">
         <is>
           <t>https://creativecommons.org/licenses/by/4.0/</t>
         </is>
       </c>
-      <c r="AA58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="13" t="inlineStr">
-        <is>
-          <t>M. abductor digiti minimi</t>
-        </is>
-      </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>untere-extremitaet</t>
-        </is>
-      </c>
-      <c r="C59" s="13" t="inlineStr">
-        <is>
-          <t>fuss</t>
-        </is>
-      </c>
-      <c r="D59" s="13" t="inlineStr">
-        <is>
-          <t>fuss,kleinzehenabduktion,kurze-fussmuskulatur,fusssohle</t>
-        </is>
-      </c>
-      <c r="E59" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="F59" s="13" t="inlineStr">
-        <is>
-          <t>Bursitis am Tuber calcanei lateral und der sog. Tailor's bunion (Prominenz des fünften Mittelfußköpfchens) gehen häufig mit Reizung des Abductor digiti minimi einher</t>
-        </is>
-      </c>
-      <c r="G59" s="13" t="inlineStr">
-        <is>
-          <t>Am lateralen Fußrand deutlich tastbar; der Muskelbauch ist von Ferse bis Kleinzehenbasis als prominenter Wulst zu verfolgen</t>
-        </is>
-      </c>
-      <c r="H59" s="13" t="inlineStr">
-        <is>
-          <t>MTP Zeh V</t>
-        </is>
-      </c>
-      <c r="I59" s="13" t="inlineStr">
-        <is>
-          <t>Zeh V: Flexion und Abduktion des MTP-Gelenks</t>
-        </is>
-      </c>
-      <c r="J59" s="13" t="inlineStr">
-        <is>
-          <t>N. tibialis (N. plantaris lateralis)</t>
-        </is>
-      </c>
-      <c r="K59" s="13" t="n"/>
-      <c r="L59" s="13" t="n"/>
-      <c r="M59" s="13" t="inlineStr">
-        <is>
-          <t>Tuber calcanei (Proc. lateralis) und Lig. plantare longum</t>
-        </is>
-      </c>
-      <c r="N59" s="13" t="n"/>
-      <c r="O59" s="13" t="n"/>
-      <c r="P59" s="13" t="n"/>
-      <c r="Q59" s="13" t="n"/>
-      <c r="R59" s="13" t="n"/>
-      <c r="S59" s="13" t="n"/>
-      <c r="T59" s="13" t="inlineStr">
-        <is>
-          <t>Zeh V, Tuberositas ossis metatarsalis V und proximale Phalanx (laterale Seite)</t>
-        </is>
-      </c>
-      <c r="U59" s="13" t="n"/>
-      <c r="V59" s="13" t="n"/>
-      <c r="W59" s="13" t="inlineStr">
-        <is>
-          <t>Abduziert und beugt die Kleinzehe im MTP-Gelenk; stabilisiert den lateralen Fußrand</t>
-        </is>
-      </c>
-      <c r="X59" s="13" t="inlineStr">
-        <is>
-          <t>BodyParts3D, © DBCLS</t>
-        </is>
-      </c>
-      <c r="Y59" s="13" t="inlineStr">
-        <is>
-          <t>CC BY 4.0</t>
-        </is>
-      </c>
-      <c r="Z59" s="13" t="inlineStr">
-        <is>
-          <t>https://creativecommons.org/licenses/by/4.0/</t>
-        </is>
-      </c>
-      <c r="AA59" s="13" t="n"/>
+      <c r="AA58" s="13" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:AA2"/>
@@ -6425,7 +6334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="41.109375" customWidth="1" style="30" min="1" max="1"/>
@@ -6543,7 +6452,7 @@
       </c>
       <c r="D5" s="17" t="inlineStr">
         <is>
-          <t>Becken: Retroversion (Dorsalkippung) im Iliosakralgelenk; Stabilisierung der LWS in Streckstellung</t>
+          <t>Kippt das Becken nach dorsal (Retroversion) und unterstützt die Stabilisierung der Lendenwirbelsäule in Streckstellung</t>
         </is>
       </c>
       <c r="E5" s="17" t="inlineStr">
@@ -6580,8 +6489,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Flexion, Adduktion, Außenrotation
-LWS (bei fixiertem Femur): Verstärkung der Lendenlordose</t>
+          <t>Beugt die Hüfte und adduziert den Oberschenkel; bei fixiertem Femur verstärkt er die Lendenlordose; wirkt zudem als Außenrotator im Hüftgelenk</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
@@ -6618,8 +6526,7 @@
       </c>
       <c r="D7" s="37" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Flexion, Außenrotation
-Becken (bei fixiertem Femur): Ventrale Beckenkippung</t>
+          <t>Flektiert das Hüftgelenk und rotiert den Oberschenkel nach außen; bei feststehendem Bein kippt er das Ilium nach ventral</t>
         </is>
       </c>
       <c r="E7" s="17" t="inlineStr">
@@ -6658,8 +6565,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Extension, Außenrotation
-Iliotibiales Band: Abduktion (laterale Anteile)</t>
+          <t>Hauptextensor des Hüftgelenks; dreht den Oberschenkel nach außen; die lateralen Anteile wirken zusätzlich als Abduktoren und spannen den Tractus iliotibialis</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
@@ -6696,9 +6602,7 @@
       </c>
       <c r="D9" s="37" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Abduktion
-Vordere Fasern: Flexion, Innenrotation
-Hintere Fasern: Extension, Außenrotation</t>
+          <t>Führt das Bein seitwärts (Abduktion); vordere Fasern rotieren nach innen und beugen, hintere Fasern rotieren nach außen und strecken; essentiell für die Beckenstabilisierung im Einbeinstand</t>
         </is>
       </c>
       <c r="E9" s="17" t="inlineStr">
@@ -6735,9 +6639,7 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Abduktion
-Ventrale Fasern: Innenrotation
-Dorsale Fasern: Außenrotation</t>
+          <t>Abduziert die Hüfte und unterstützt die Innenrotation (ventrale Fasern) bzw. Außenrotation (dorsale Fasern); Funktion nahezu identisch mit Gluteus medius</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
@@ -6774,7 +6676,7 @@
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Adduktion, Flexion, Außenrotation</t>
+          <t>Adduziert den Oberschenkel und beugt ihn leicht im Hüftgelenk; eine geringe Außenrotation ist ebenfalls möglich</t>
         </is>
       </c>
       <c r="E11" s="17" t="inlineStr">
@@ -6811,7 +6713,7 @@
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Adduktion, Flexion, Außenrotation</t>
+          <t>Führt den Oberschenkel zur Körpermitte (Adduktion); unterstützt zugleich die Hüftbeugung und eine leichte Außenrotation</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
@@ -6848,7 +6750,7 @@
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Adduktion, Flexion, Außenrotation</t>
+          <t>Führt den Oberschenkel zur Körpermitte (Adduktion); unterstützt zugleich die Hüftbeugung und eine leichte Außenrotation</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
@@ -6889,9 +6791,7 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Adduktion
-Pubischer Anteil: Flexion, Außenrotation
-Ischiokruraler Anteil: Extension, Innenrotation</t>
+          <t>Kräftiger Adduktor des Hüftgelenks; streckt die Hüfte (insbesondere der ischiokrurale Anteil); der pubische Anteil rotiert nach außen, der ischiokrurale Anteil nach innen</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
@@ -6928,8 +6828,7 @@
       </c>
       <c r="D15" s="37" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Außenrotation
-Bei 90° Flexion: zusätzlich Abduktion</t>
+          <t>Außenrotiert den Oberschenkel im Hüftgelenk; wirkt bei 90° Hüftbeugung zusätzlich als Abduktor</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
@@ -6966,7 +6865,7 @@
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Außenrotation</t>
+          <t>Dreht den Oberschenkel im Hüftgelenk nach außen</t>
         </is>
       </c>
       <c r="E16" s="18" t="inlineStr">
@@ -7003,7 +6902,7 @@
       </c>
       <c r="D17" s="17" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Außenrotation</t>
+          <t>Dreht den Oberschenkel im Hüftgelenk nach außen</t>
         </is>
       </c>
       <c r="E17" s="17" t="inlineStr">
@@ -7040,7 +6939,7 @@
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Außenrotation</t>
+          <t>Unterstützt die Außenrotation im Hüftgelenk</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
@@ -7077,7 +6976,7 @@
       </c>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Außenrotation</t>
+          <t>Unterstützt die Außenrotation im Hüftgelenk</t>
         </is>
       </c>
       <c r="E19" s="17" t="inlineStr">
@@ -7114,7 +7013,7 @@
       </c>
       <c r="D20" s="18" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Außenrotation, Adduktion</t>
+          <t>Dreht den Oberschenkel nach außen und zieht ihn leicht zur Körpermitte (Adduktion); liegt zwischen Tuber ischiadicum und Crista intertrochanterica</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
@@ -7151,8 +7050,7 @@
       </c>
       <c r="D21" s="37" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Abduktion, Flexion, Innenrotation
-Kniegelenk (Art. genus): Flexion, Spannung des Tractus iliotibialis</t>
+          <t>Abduziert und beugt die Hüfte, dreht den Oberschenkel nach innen; spannt den Tractus iliotibialis und entlastet damit Femurschaft und -hals</t>
         </is>
       </c>
       <c r="E21" s="17" t="inlineStr">
@@ -7189,8 +7087,7 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Flexion, Außenrotation, Abduktion
-Kniegelenk (Art. genus): Flexion, Innenrotation des Unterschenkels</t>
+          <t>Beugt und dreht die Hüfte nach außen; abduziert; im Kniegelenk bewirkt er Beugung und Innenrotation des Unterschenkels – typische Schneidersitzposition</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
@@ -7227,8 +7124,7 @@
       </c>
       <c r="D23" s="37" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Adduktion
-Kniegelenk (Art. genus): Flexion, Innenrotation des Unterschenkels</t>
+          <t>Adduziert das Bein im Hüftgelenk; im Kniegelenk wirkt er als Beuger und Innenrotator des Unterschenkels</t>
         </is>
       </c>
       <c r="E23" s="17" t="inlineStr">
@@ -7272,9 +7168,7 @@
       </c>
       <c r="D25" s="38" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Flexion
-Kniegelenk (Art. genus): Extension
-(Einziger zweigelenkiger Quadricepsanteil)</t>
+          <t>Beugt die Hüfte im Hüftgelenk (Flexion in der Art. coxae); streckt das Kniegelenk als Teil des Quadriceps (Extension in der Art. genus)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -7312,9 +7206,7 @@
       </c>
       <c r="D26" s="22" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Extension
-Kniegelenk (Art. genus): Flexion
-Bei gebeugtem Knie: Außenrotation des Unterschenkels</t>
+          <t>Streckt die Hüfte (Extension in der Art. coxae) und beugt das Knie (Flexion in der Art. genus); bei gebeugtem Knie Außenrotation des Unterschenkels</t>
         </is>
       </c>
       <c r="E26" s="21" t="inlineStr">
@@ -7351,9 +7243,7 @@
       </c>
       <c r="D27" s="38" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Extension
-Kniegelenk (Art. genus): Flexion
-Bei gebeugtem Knie: Innenrotation des Unterschenkels</t>
+          <t>Streckt die Hüfte (Extension in der Art. coxae) und beugt das Knie (Flexion in der Art. genus); bei gebeugtem Knie Innenrotation des Unterschenkels</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -7391,9 +7281,7 @@
       </c>
       <c r="D28" s="22" t="inlineStr">
         <is>
-          <t>Hüftgelenk (Art. coxae): Extension
-Kniegelenk (Art. genus): Flexion
-Bei gebeugtem Knie: Innenrotation des Unterschenkels</t>
+          <t>Streckt die Hüfte (Extension in der Art. coxae) und beugt das Knie (Flexion in der Art. genus); bei gebeugtem Knie Innenrotation des Unterschenkels; zieht den Meniscus lateralis nach dorsal</t>
         </is>
       </c>
       <c r="E28" s="21" t="inlineStr">
@@ -7430,8 +7318,7 @@
       </c>
       <c r="D29" s="38" t="inlineStr">
         <is>
-          <t>Kniegelenk (Art. genus): Extension
-Patellamediale Stabilisierung (VMO-Anteil)</t>
+          <t>Streckt das Knie (Extension in der Art. genus); der schräg verlaufende distale Anteil (VMO) stabilisiert die Patella nach medial</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -7468,7 +7355,7 @@
       </c>
       <c r="D30" s="21" t="inlineStr">
         <is>
-          <t>Kniegelenk (Art. genus): Extension</t>
+          <t>Streckt das Knie (Extension in der Art. genus); bildet gemeinsam mit den anderen Quadricepsanteilen die Hauptkraft für die Knieextension</t>
         </is>
       </c>
       <c r="E30" s="21" t="inlineStr">
@@ -7505,7 +7392,7 @@
       </c>
       <c r="D31" s="20" t="inlineStr">
         <is>
-          <t>Kniegelenk (Art. genus): Extension</t>
+          <t>Streckt das Knie (Extension in der Art. genus); beeinflusst die Patellastellung über das laterale Retinaculum</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -7542,8 +7429,7 @@
       </c>
       <c r="D32" s="22" t="inlineStr">
         <is>
-          <t>Kniegelenk (Art. genus): Flexion
-Bei gebeugtem Knie: Außenrotation des Unterschenkels</t>
+          <t>Beugt das Knie (Flexion in der Art. genus); dreht den Unterschenkel bei gebeugtem Knie nach außen (Außenrotation)</t>
         </is>
       </c>
       <c r="E32" s="21" t="inlineStr">
@@ -7580,7 +7466,7 @@
       </c>
       <c r="D33" s="20" t="inlineStr">
         <is>
-          <t>Kniegelenk (Art. genus): Spannung des Recessus suprapatellaris (verhindert Kapsel-Einklemmen bei Streckung)</t>
+          <t>Spannt die Kniegelenkkapsel im Recessus suprapatellaris (verhindert Einklemmen bei Kniestreckung)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -7617,7 +7503,7 @@
       </c>
       <c r="D34" s="21" t="inlineStr">
         <is>
-          <t>Kniegelenk (Art. genus): Flexion, Innenrotation des Unterschenkels (Entriegelung aus Vollextension)</t>
+          <t>Leitet die Kniebeugung ein, rotiert den Unterschenkel nach innen und entlastet den Außenmeniskus</t>
         </is>
       </c>
       <c r="E34" s="21" t="inlineStr">
@@ -7746,7 +7632,7 @@
       </c>
       <c r="F38" s="23" t="inlineStr">
         <is>
-          <t>Fehlt bei etwa 15 % der Bevölkerung; seine dünne Sehne ist als Transplantatmaterial beliebt (z.B. für Bandrekonstruktionen); klinisch selten symptomatisch</t>
+          <t>Der Muskel fehlt bei vielen Menschen ganz; meist bleibt das ohne Beschwerden, die Sehne wird aber teils als Transplantat genutzt</t>
         </is>
       </c>
       <c r="G38" s="23" t="inlineStr">
@@ -8145,7 +8031,7 @@
       </c>
       <c r="D49" s="25" t="inlineStr">
         <is>
-          <t>Richtet den Zugvektor des M. flexor digitorum longus auf die Zehenlängsachse aus; unterstützt die Beugung der Zehen II–V</t>
+          <t>Richtet die Zugrichtung des langen Zehenbeugers aus und unterstützt das Beugen der Kleinzehen</t>
         </is>
       </c>
       <c r="E49" s="25" t="inlineStr">
@@ -8155,7 +8041,7 @@
       </c>
       <c r="F49" s="25" t="inlineStr">
         <is>
-          <t>Korrigiert den durch den Zug des M. flexor digitorum longus entstehenden schrägen Zugvektor; erst durch ihn erfolgt eine achsengerechte Zehenflexion</t>
+          <t>Verbessert die Kraftübertragung auf die Kleinzehen; Schwäche macht die plantare Zehenbeugung weniger sauber</t>
         </is>
       </c>
       <c r="G49" s="25" t="inlineStr">
@@ -8293,7 +8179,7 @@
       </c>
       <c r="D53" s="25" t="inlineStr">
         <is>
-          <t>Streckt die Großzehe im MTP-Gelenk; unterstützt den M. extensor hallucis longus bei der Großzehenstreckung</t>
+          <t>Streckt die Großzehe im Grundgelenk und unterstützt die lange Strecksehne</t>
         </is>
       </c>
       <c r="E53" s="25" t="inlineStr">
@@ -8463,69 +8349,37 @@
       </c>
     </row>
     <row r="58" ht="45" customHeight="1" s="30">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>M. opponens digiti minimi</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Lig. plantare longum, Basis des Os metatarsale V und Sehnenscheide des M. fibularis longus</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Lateraler Rand des Os metatarsale V</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Unterstützt Flexion und Abduktion der Kleinzehe und stabilisiert das laterale Längsgewölbe des Fußes</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>N. tibialis (N. plantaris lateralis), S2, S3</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Wird oft nur als tiefer Anteil des M. flexor digiti minimi brevis beschrieben und daher in Lehrwerken nicht immer separat aufgeführt; funktionell trägt er zur Stabilisierung des lateralen Fußrandes bei</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="23" t="inlineStr">
+      <c r="A58" s="23" t="inlineStr">
         <is>
           <t>M. abductor digiti minimi</t>
         </is>
       </c>
-      <c r="B59" s="23" t="inlineStr">
+      <c r="B58" s="23" t="inlineStr">
         <is>
           <t>Tuber calcanei (Proc. lateralis) und Lig. plantare longum</t>
         </is>
       </c>
-      <c r="C59" s="23" t="inlineStr">
+      <c r="C58" s="23" t="inlineStr">
         <is>
           <t>Zeh V, Tuberositas ossis metatarsalis V und proximale Phalanx (laterale Seite)</t>
         </is>
       </c>
-      <c r="D59" s="23" t="inlineStr">
+      <c r="D58" s="23" t="inlineStr">
         <is>
           <t>Abduziert und beugt die Kleinzehe im MTP-Gelenk; stabilisiert den lateralen Fußrand</t>
         </is>
       </c>
-      <c r="E59" s="23" t="inlineStr">
+      <c r="E58" s="23" t="inlineStr">
         <is>
           <t>N. tibialis (N. plantaris lateralis)</t>
         </is>
       </c>
-      <c r="F59" s="23" t="inlineStr">
+      <c r="F58" s="23" t="inlineStr">
         <is>
           <t>Bursitis am Tuber calcanei lateral und der sog. Tailor's bunion (Prominenz des fünften Mittelfußköpfchens) gehen häufig mit Reizung des Abductor digiti minimi einher</t>
         </is>
       </c>
-      <c r="G59" s="23" t="inlineStr">
+      <c r="G58" s="23" t="inlineStr">
         <is>
           <t>Am lateralen Fußrand deutlich tastbar; der Muskelbauch ist von Ferse bis Kleinzehenbasis als prominenter Wulst zu verfolgen</t>
         </is>

</xml_diff>